<commit_message>
feat: update background and transition generators with new translation types and formatting; enhance voice generator parameter handling
</commit_message>
<xml_diff>
--- a/param_config/param_data_renpy.xlsx
+++ b/param_config/param_data_renpy.xlsx
@@ -1,38 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\视觉小说项目\【表格演出工具】dev\param_config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\视觉小说项目\【表格演出工具】git仓库\param_config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD303094-E6C7-456E-B22C-9D3A07F8A70C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683CE365-FB8E-4835-A0C7-9CD54F377FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Command" sheetId="16" r:id="rId1"/>
     <sheet name="Layer" sheetId="1" r:id="rId2"/>
-    <sheet name="Transform" sheetId="2" r:id="rId3"/>
-    <sheet name="Transition" sheetId="3" r:id="rId4"/>
-    <sheet name="Camera" sheetId="20" r:id="rId5"/>
-    <sheet name="Name" sheetId="5" r:id="rId6"/>
-    <sheet name="Character" sheetId="11" r:id="rId7"/>
-    <sheet name="Sprite" sheetId="17" r:id="rId8"/>
-    <sheet name="Varient" sheetId="15" r:id="rId9"/>
-    <sheet name="ATLtype" sheetId="18" r:id="rId10"/>
-    <sheet name="Warp" sheetId="19" r:id="rId11"/>
-    <sheet name="Animation" sheetId="12" r:id="rId12"/>
-    <sheet name="Background" sheetId="6" r:id="rId13"/>
-    <sheet name="Event" sheetId="7" r:id="rId14"/>
-    <sheet name="Movie" sheetId="10" r:id="rId15"/>
-    <sheet name="Music" sheetId="8" r:id="rId16"/>
-    <sheet name="Ambience" sheetId="14" r:id="rId17"/>
-    <sheet name="Sound" sheetId="9" r:id="rId18"/>
-    <sheet name="Window" sheetId="13" r:id="rId19"/>
-    <sheet name="基础参数模板" sheetId="4" r:id="rId20"/>
+    <sheet name="BackTransform" sheetId="21" r:id="rId3"/>
+    <sheet name="Transform" sheetId="2" r:id="rId4"/>
+    <sheet name="Transition" sheetId="3" r:id="rId5"/>
+    <sheet name="Camera" sheetId="20" r:id="rId6"/>
+    <sheet name="Name" sheetId="5" r:id="rId7"/>
+    <sheet name="Character" sheetId="11" r:id="rId8"/>
+    <sheet name="Sprite" sheetId="17" r:id="rId9"/>
+    <sheet name="Varient" sheetId="15" r:id="rId10"/>
+    <sheet name="ATLtype" sheetId="18" r:id="rId11"/>
+    <sheet name="Warp" sheetId="19" r:id="rId12"/>
+    <sheet name="Animation" sheetId="12" r:id="rId13"/>
+    <sheet name="Background" sheetId="6" r:id="rId14"/>
+    <sheet name="Event" sheetId="7" r:id="rId15"/>
+    <sheet name="Movie" sheetId="10" r:id="rId16"/>
+    <sheet name="Music" sheetId="8" r:id="rId17"/>
+    <sheet name="Ambience" sheetId="14" r:id="rId18"/>
+    <sheet name="Sound" sheetId="9" r:id="rId19"/>
+    <sheet name="Window" sheetId="13" r:id="rId20"/>
+    <sheet name="基础参数模板" sheetId="4" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="85">
   <si>
     <t>master</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -381,6 +382,14 @@
   </si>
   <si>
     <t>None</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>背景变换</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>the_back_transform</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -721,9 +730,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE878D2C-D55B-43FC-94A3-38F8F06D95DD}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -775,11 +784,43 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2EE69BF-A36D-4600-8BBD-F190242D61E1}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A408B64A-B708-430C-BB8C-9D370F261E67}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -854,12 +895,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1F7FAF2-D815-4AEE-98A8-BF63C30F7270}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -910,12 +951,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E58EBDF9-D3A0-47BB-830B-8DFDC52004A0}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -942,12 +983,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C90C90F-14F7-48DC-A223-3A21F823BBD9}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -982,12 +1023,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D0F9688-485C-4089-A924-659F7B17ED40}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1014,12 +1055,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F2FB37-B05C-42DD-AD48-6F5711AA0F97}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1046,12 +1087,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4D0EA6C-94B5-4B28-9D79-AE5F33D06CF7}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1086,12 +1127,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEACBE5A-FAED-480E-A890-20FE9FA50E67}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1126,12 +1167,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{966183FE-893C-4CE5-91A9-7B2DDB5030D5}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1166,12 +1207,52 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B88F63F-8C77-4EB4-9A0D-787BFC3AC2C7}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1205,52 +1286,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD06AC-723F-4A84-9034-732CCFF1C997}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1270,11 +1311,46 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19CFEAC7-C64A-4C93-A38C-C48313C3D5D4}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1325,12 +1401,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1389,12 +1465,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{265D460B-FFAA-4C4F-A951-71A95CD67F62}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1445,12 +1521,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{938A5E86-0F35-431D-B760-B491C7011A1E}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1477,12 +1553,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B366D178-7CDC-4708-83DB-8F05B13E7EF6}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1509,12 +1585,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F873D92-1EFE-4746-B5A3-015962221CAC}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1539,36 +1615,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2EE69BF-A36D-4600-8BBD-F190242D61E1}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-</worksheet>
 </file>
</xml_diff>